<commit_message>
add maintenance batch alert for Sunday and Wednesday duties
Appends 'You have to run MAINTENANCE BATCH today.' to TODAY email
body when duty falls on Sunday or Wednesday. No change for other
days or for tomorrow reminder emails.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RoasterList.xlsx
+++ b/RoasterList.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\All Projects\CMS-GIT\RoasterAlert\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\DPDC Stuff\CMS-GIT\RoasterAlert\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07E9EB04-EB20-42BB-AD26-EA16B8B611AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A971F7A-A1B0-4715-BE1B-6E8ECC2E8612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D1ADB46A-FEE1-453A-9125-EB62AA815D9C}"/>
   </bookViews>

</xml_diff>